<commit_message>
changes in generate-xml to take read path in consideration
</commit_message>
<xml_diff>
--- a/spreadsheet_template.xlsx
+++ b/spreadsheet_template.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="project" sheetId="1" state="visible" r:id="rId3"/>
@@ -64,6 +64,18 @@
         </r>
       </text>
     </comment>
+    <comment ref="D1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">free text</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -537,11 +549,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="71">
   <si>
     <t xml:space="preserve">Project ID</t>
   </si>
   <si>
+    <t xml:space="preserve">Name</t>
+  </si>
+  <si>
     <t xml:space="preserve">Title</t>
   </si>
   <si>
@@ -549,6 +564,9 @@
   </si>
   <si>
     <t xml:space="preserve">proj_0000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yeasts from Lunar soils</t>
   </si>
   <si>
     <t xml:space="preserve">Diversity of yeast isolated from Lunar soils</t>
@@ -1079,12 +1097,12 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15.25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="78.91"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="78.91"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1097,16 +1115,22 @@
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -1146,101 +1170,101 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>4932</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C3" s="1" t="n">
         <v>4932</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -1263,7 +1287,7 @@
   <dimension ref="A1:P6"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.8"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="49.32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="15.7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12.9"/>
@@ -1283,87 +1307,87 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="M1" s="7" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="K2" s="7" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="L2" s="7" t="n">
         <v>300</v>
@@ -1372,48 +1396,48 @@
         <v>30</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="P2" s="1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="L3" s="7" t="n">
         <v>300</v>
@@ -1422,13 +1446,13 @@
         <v>30</v>
       </c>
       <c r="N3" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1486,53 +1510,53 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>